<commit_message>
backup: 2026-08-30 23:33:35 (9140 paths)
</commit_message>
<xml_diff>
--- a/game_specs.xlsx
+++ b/game_specs.xlsx
@@ -2652,32 +2652,32 @@
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>圖鑑CG</t>
+          <t>切西瓜</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>swimsuit_default</t>
+          <t>stock_accumulate</t>
         </is>
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>夏日祭・清涼泳裝</t>
+          <t>自動刷關切西瓜累計</t>
         </is>
       </c>
       <c r="D5" t="inlineStr">
         <is>
-          <t>預設泳裝立繪</t>
+          <t>勝場自動累積 +1 (上限 999 次)</t>
         </is>
       </c>
       <c r="E5" t="inlineStr">
         <is>
-          <t>通關第 1 關或觸發泳裝事件</t>
+          <t>多輪連續挑戰</t>
         </is>
       </c>
       <c r="F5" t="inlineStr">
         <is>
-          <t>小樂難得換上的清涼泳裝</t>
+          <t>自動刷關開啟獨立浮動面板，無全屏遮罩，隨時暫停/繼續，三階段重複挑戰</t>
         </is>
       </c>
     </row>
@@ -2689,25 +2689,57 @@
       </c>
       <c r="B6" t="inlineStr">
         <is>
+          <t>swimsuit_default</t>
+        </is>
+      </c>
+      <c r="C6" t="inlineStr">
+        <is>
+          <t>夏日祭・清涼泳裝</t>
+        </is>
+      </c>
+      <c r="D6" t="inlineStr">
+        <is>
+          <t>預設泳裝立繪</t>
+        </is>
+      </c>
+      <c r="E6" t="inlineStr">
+        <is>
+          <t>通關第 1 關或觸發泳裝事件</t>
+        </is>
+      </c>
+      <c r="F6" t="inlineStr">
+        <is>
+          <t>小樂難得換上的清涼泳裝</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>圖鑑CG</t>
+        </is>
+      </c>
+      <c r="B7" t="inlineStr">
+        <is>
           <t>swimsuit_watermelon</t>
         </is>
       </c>
-      <c r="C6" t="inlineStr">
+      <c r="C7" t="inlineStr">
         <is>
           <t>海風・切西瓜</t>
         </is>
       </c>
-      <c r="D6" t="inlineStr">
+      <c r="D7" t="inlineStr">
         <is>
           <t>切西瓜差分立繪</t>
         </is>
       </c>
-      <c r="E6" t="inlineStr">
+      <c r="E7" t="inlineStr">
         <is>
           <t>完成蒙眼切西瓜大挑戰</t>
         </is>
       </c>
-      <c r="F6" t="inlineStr">
+      <c r="F7" t="inlineStr">
         <is>
           <t>蒙眼切西瓜大獲全勝後，小樂得意洋洋展示成果的模樣</t>
         </is>
@@ -2792,12 +2824,12 @@
       </c>
       <c r="D3" t="inlineStr">
         <is>
-          <t>Level, XP, SP, Coins, Potions, Allocations</t>
+          <t>Level, XP, SP, Coins, Potions, Allocations, WatermelonStock</t>
         </is>
       </c>
       <c r="E3" t="inlineStr">
         <is>
-          <t>任意修改玩家等級、金幣、藥水與點數分配</t>
+          <t>任意修改玩家等級、金幣、藥水、點數分配與切西瓜庫存</t>
         </is>
       </c>
     </row>
@@ -3324,133 +3356,214 @@
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>ui.clearAll</t>
+          <t>ui.autoWatermelonStock</t>
         </is>
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>ui.clearAll</t>
+          <t>累計切西瓜次數：5 / 999</t>
         </is>
       </c>
       <c r="C18" t="inlineStr">
         <is>
-          <t>ui.clearAll</t>
+          <t>累計切西瓜次數：5 / 999</t>
         </is>
       </c>
       <c r="D18" t="inlineStr">
         <is>
-          <t>ui.clearAll</t>
+          <t>累計切西瓜次數：5 / 999</t>
         </is>
       </c>
       <c r="E18" t="inlineStr">
         <is>
-          <t>ui.clearAll</t>
+          <t>累計切西瓜次數：5 / 999</t>
         </is>
       </c>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>ui.equip</t>
+          <t>ui.btnNextWatermelonRound</t>
         </is>
       </c>
       <c r="B19" t="inlineStr">
         <is>
-          <t>ui.equip</t>
+          <t>進行下一輪切西瓜 (剩餘 5)</t>
         </is>
       </c>
       <c r="C19" t="inlineStr">
         <is>
-          <t>ui.equip</t>
+          <t>進行下一輪切西瓜 (剩餘 5)</t>
         </is>
       </c>
       <c r="D19" t="inlineStr">
         <is>
-          <t>ui.equip</t>
+          <t>進行下一輪切西瓜 (剩餘 5)</t>
         </is>
       </c>
       <c r="E19" t="inlineStr">
         <is>
-          <t>ui.equip</t>
+          <t>進行下一輪切西瓜 (剩餘 5)</t>
         </is>
       </c>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>ui.unequip</t>
+          <t>ui.floatingWatermelonTitle</t>
         </is>
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>ui.unequip</t>
+          <t>🍉 蒙眼切西瓜 (自動刷關累積)</t>
         </is>
       </c>
       <c r="C20" t="inlineStr">
         <is>
-          <t>ui.unequip</t>
+          <t>🍉 蒙眼切西瓜 (自動刷關累積)</t>
         </is>
       </c>
       <c r="D20" t="inlineStr">
         <is>
-          <t>ui.unequip</t>
+          <t>🍉 蒙眼切西瓜 (自動刷關累積)</t>
         </is>
       </c>
       <c r="E20" t="inlineStr">
         <is>
-          <t>ui.unequip</t>
+          <t>🍉 蒙眼切西瓜 (自動刷關累積)</t>
         </is>
       </c>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>ui.victory</t>
+          <t>ui.clearAll</t>
         </is>
       </c>
       <c r="B21" t="inlineStr">
         <is>
-          <t>ui.victory</t>
+          <t>ui.clearAll</t>
         </is>
       </c>
       <c r="C21" t="inlineStr">
         <is>
-          <t>ui.victory</t>
+          <t>ui.clearAll</t>
         </is>
       </c>
       <c r="D21" t="inlineStr">
         <is>
-          <t>ui.victory</t>
+          <t>ui.clearAll</t>
         </is>
       </c>
       <c r="E21" t="inlineStr">
         <is>
-          <t>ui.victory</t>
+          <t>ui.clearAll</t>
         </is>
       </c>
     </row>
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
+          <t>ui.equip</t>
+        </is>
+      </c>
+      <c r="B22" t="inlineStr">
+        <is>
+          <t>ui.equip</t>
+        </is>
+      </c>
+      <c r="C22" t="inlineStr">
+        <is>
+          <t>ui.equip</t>
+        </is>
+      </c>
+      <c r="D22" t="inlineStr">
+        <is>
+          <t>ui.equip</t>
+        </is>
+      </c>
+      <c r="E22" t="inlineStr">
+        <is>
+          <t>ui.equip</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" t="inlineStr">
+        <is>
+          <t>ui.unequip</t>
+        </is>
+      </c>
+      <c r="B23" t="inlineStr">
+        <is>
+          <t>ui.unequip</t>
+        </is>
+      </c>
+      <c r="C23" t="inlineStr">
+        <is>
+          <t>ui.unequip</t>
+        </is>
+      </c>
+      <c r="D23" t="inlineStr">
+        <is>
+          <t>ui.unequip</t>
+        </is>
+      </c>
+      <c r="E23" t="inlineStr">
+        <is>
+          <t>ui.unequip</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" t="inlineStr">
+        <is>
+          <t>ui.victory</t>
+        </is>
+      </c>
+      <c r="B24" t="inlineStr">
+        <is>
+          <t>ui.victory</t>
+        </is>
+      </c>
+      <c r="C24" t="inlineStr">
+        <is>
+          <t>ui.victory</t>
+        </is>
+      </c>
+      <c r="D24" t="inlineStr">
+        <is>
+          <t>ui.victory</t>
+        </is>
+      </c>
+      <c r="E24" t="inlineStr">
+        <is>
+          <t>ui.victory</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" t="inlineStr">
+        <is>
           <t>ui.defeat</t>
         </is>
       </c>
-      <c r="B22" t="inlineStr">
+      <c r="B25" t="inlineStr">
         <is>
           <t>ui.defeat</t>
         </is>
       </c>
-      <c r="C22" t="inlineStr">
+      <c r="C25" t="inlineStr">
         <is>
           <t>ui.defeat</t>
         </is>
       </c>
-      <c r="D22" t="inlineStr">
+      <c r="D25" t="inlineStr">
         <is>
           <t>ui.defeat</t>
         </is>
       </c>
-      <c r="E22" t="inlineStr">
+      <c r="E25" t="inlineStr">
         <is>
           <t>ui.defeat</t>
         </is>

</xml_diff>

<commit_message>
feat(save-records): add save seed code management, cross-device transfer modal and danger zone save reset
</commit_message>
<xml_diff>
--- a/game_specs.xlsx
+++ b/game_specs.xlsx
@@ -9,7 +9,7 @@
     <sheet name="戰鬥與QTE規則" sheetId="5" r:id="rId5"/>
     <sheet name="成長與數值公式" sheetId="6" r:id="rId6"/>
     <sheet name="切西瓜與圖鑑" sheetId="7" r:id="rId7"/>
-    <sheet name="作弊與除錯" sheetId="8" r:id="rId8"/>
+    <sheet name="存檔與作弊管理" sheetId="8" r:id="rId8"/>
     <sheet name="在地化字典" sheetId="9" r:id="rId9"/>
   </sheets>
 </workbook>
@@ -2760,12 +2760,12 @@
       </c>
       <c r="B1" t="inlineStr">
         <is>
-          <t>觸發方式</t>
+          <t>觸發/操作方式</t>
         </is>
       </c>
       <c r="C1" t="inlineStr">
         <is>
-          <t>時間窗口</t>
+          <t>格式/時間窗口</t>
         </is>
       </c>
       <c r="D1" t="inlineStr">
@@ -2782,106 +2782,214 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>秘密作弊面板</t>
+          <t>存檔種子碼導出</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>連續按下 4 次數字鍵 8</t>
+          <t>點擊首頁【💾 存檔紀錄】彈窗</t>
         </is>
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>1000ms 滾動窗口</t>
+          <t>KORAKU1_&lt;Base64UTF8JSON&gt;</t>
         </is>
       </c>
       <c r="D2" t="inlineStr">
         <is>
-          <t>主鍵區 8 或小鍵盤 8</t>
+          <t>一鍵複製種子碼</t>
         </is>
       </c>
       <c r="E2" t="inlineStr">
         <is>
-          <t>彈出作弊設定面板，可自訂全部存檔資料</t>
+          <t>將玩家當前等級、經驗、SP、星砂、12格裝備、背包、技能與戰績完整導出為字串</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>自訂屬性數值</t>
+          <t>存檔種子碼匯入</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>作弊面板輸入數值</t>
+          <t>貼上種子碼並點擊【載入並套用】</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>即時套用</t>
+          <t>驗證格式與合法性</t>
         </is>
       </c>
       <c r="D3" t="inlineStr">
         <is>
-          <t>Level, XP, SP, Coins, Potions, Allocations, WatermelonStock</t>
+          <t>覆蓋當前存檔進度</t>
         </is>
       </c>
       <c r="E3" t="inlineStr">
         <is>
-          <t>任意修改玩家等級、金幣、藥水、點數分配與切西瓜庫存</t>
+          <t>跨設備/瀏覽器轉移遊戲紀錄，自動寫入 localStorage 並刷新全域畫面</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>一鍵解鎖全關卡</t>
+          <t>重置存檔</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>作弊面板點擊按鈕</t>
+          <t>存檔紀錄彈窗底部【危險區域】</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>即時套用</t>
+          <t>彈出確認對話框</t>
         </is>
       </c>
       <c r="D4" t="inlineStr">
         <is>
-          <t>clearedStages: [1, 2, 3, 4]</t>
+          <t>清除全部資料回歸初始狀態</t>
         </is>
       </c>
       <c r="E4" t="inlineStr">
         <is>
-          <t>直接解鎖全 4 大章節關卡與 Boss 規則說明卡</t>
+          <t>清空等級、星砂、裝備、技能與戰績紀錄，回歸 Lv.1 初始角色</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
+          <t>秘密作弊面板</t>
+        </is>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>連續按下 4 次數字鍵 8</t>
+        </is>
+      </c>
+      <c r="C5" t="inlineStr">
+        <is>
+          <t>1000ms 滾動窗口</t>
+        </is>
+      </c>
+      <c r="D5" t="inlineStr">
+        <is>
+          <t>主鍵區 8 或小鍵盤 8</t>
+        </is>
+      </c>
+      <c r="E5" t="inlineStr">
+        <is>
+          <t>彈出作弊設定面板，可自訂全部存檔資料</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>作弊密碼驗證</t>
+        </is>
+      </c>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>首頁點擊【⚙️ 測試調試 / 作弊選單】</t>
+        </is>
+      </c>
+      <c r="C6" t="inlineStr">
+        <is>
+          <t>輸入密碼 8989</t>
+        </is>
+      </c>
+      <c r="D6" t="inlineStr">
+        <is>
+          <t>解鎖作弊選單</t>
+        </is>
+      </c>
+      <c r="E6" t="inlineStr">
+        <is>
+          <t>防止誤觸，驗證成功後開啟作弊面板</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>自訂屬性數值</t>
+        </is>
+      </c>
+      <c r="B7" t="inlineStr">
+        <is>
+          <t>作弊面板輸入數值</t>
+        </is>
+      </c>
+      <c r="C7" t="inlineStr">
+        <is>
+          <t>即時套用</t>
+        </is>
+      </c>
+      <c r="D7" t="inlineStr">
+        <is>
+          <t>Level, XP, SP, Coins, Potions, Allocations, Skills</t>
+        </is>
+      </c>
+      <c r="E7" t="inlineStr">
+        <is>
+          <t>任意修改玩家等級、金幣、藥水、點數分配與技能</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>一鍵解鎖全關卡</t>
+        </is>
+      </c>
+      <c r="B8" t="inlineStr">
+        <is>
+          <t>作弊面板點擊按鈕</t>
+        </is>
+      </c>
+      <c r="C8" t="inlineStr">
+        <is>
+          <t>即時套用</t>
+        </is>
+      </c>
+      <c r="D8" t="inlineStr">
+        <is>
+          <t>clearedStages: [1, 2, 3, 4]</t>
+        </is>
+      </c>
+      <c r="E8" t="inlineStr">
+        <is>
+          <t>直接解鎖全 4 大章節關卡與 Boss 規則說明卡</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
           <t>一鍵解鎖全圖鑑</t>
         </is>
       </c>
-      <c r="B5" t="inlineStr">
+      <c r="B9" t="inlineStr">
         <is>
           <t>作弊面板點擊按鈕</t>
         </is>
       </c>
-      <c r="C5" t="inlineStr">
+      <c r="C9" t="inlineStr">
         <is>
           <t>即時套用</t>
         </is>
       </c>
-      <c r="D5" t="inlineStr">
-        <is>
-          <t>unlockedSwimsuit: true</t>
-        </is>
-      </c>
-      <c r="E5" t="inlineStr">
+      <c r="D9" t="inlineStr">
+        <is>
+          <t>unlockedSwimsuit: true, unlockedGalleryAll: true</t>
+        </is>
+      </c>
+      <c r="E9" t="inlineStr">
         <is>
           <t>立即解鎖全部泳裝與切西瓜立繪圖鑑</t>
         </is>
@@ -3569,6 +3677,141 @@
         </is>
       </c>
     </row>
+    <row r="26">
+      <c r="A26" t="inlineStr">
+        <is>
+          <t>ui.saveRecord</t>
+        </is>
+      </c>
+      <c r="B26" t="inlineStr">
+        <is>
+          <t>💾 存檔紀錄</t>
+        </is>
+      </c>
+      <c r="C26" t="inlineStr">
+        <is>
+          <t>💾 存檔紀錄</t>
+        </is>
+      </c>
+      <c r="D26" t="inlineStr">
+        <is>
+          <t>💾 存檔紀錄</t>
+        </is>
+      </c>
+      <c r="E26" t="inlineStr">
+        <is>
+          <t>💾 存檔紀錄</t>
+        </is>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" t="inlineStr">
+        <is>
+          <t>ui.saveRecordModalTitle</t>
+        </is>
+      </c>
+      <c r="B27" t="inlineStr">
+        <is>
+          <t>💾 存檔紀錄與種子碼管理</t>
+        </is>
+      </c>
+      <c r="C27" t="inlineStr">
+        <is>
+          <t>💾 存檔紀錄與種子碼管理</t>
+        </is>
+      </c>
+      <c r="D27" t="inlineStr">
+        <is>
+          <t>💾 存檔紀錄與種子碼管理</t>
+        </is>
+      </c>
+      <c r="E27" t="inlineStr">
+        <is>
+          <t>💾 存檔紀錄與種子碼管理</t>
+        </is>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" t="inlineStr">
+        <is>
+          <t>ui.btnCopySaveSeed</t>
+        </is>
+      </c>
+      <c r="B28" t="inlineStr">
+        <is>
+          <t>📋 複製種子碼</t>
+        </is>
+      </c>
+      <c r="C28" t="inlineStr">
+        <is>
+          <t>📋 複製種子碼</t>
+        </is>
+      </c>
+      <c r="D28" t="inlineStr">
+        <is>
+          <t>📋 複製種子碼</t>
+        </is>
+      </c>
+      <c r="E28" t="inlineStr">
+        <is>
+          <t>📋 複製種子碼</t>
+        </is>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" t="inlineStr">
+        <is>
+          <t>ui.btnImportSaveSeed</t>
+        </is>
+      </c>
+      <c r="B29" t="inlineStr">
+        <is>
+          <t>📥 載入並套用種子碼</t>
+        </is>
+      </c>
+      <c r="C29" t="inlineStr">
+        <is>
+          <t>📥 載入並套用種子碼</t>
+        </is>
+      </c>
+      <c r="D29" t="inlineStr">
+        <is>
+          <t>📥 載入並套用種子碼</t>
+        </is>
+      </c>
+      <c r="E29" t="inlineStr">
+        <is>
+          <t>📥 載入並套用種子碼</t>
+        </is>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" t="inlineStr">
+        <is>
+          <t>ui.btnModalResetSave</t>
+        </is>
+      </c>
+      <c r="B30" t="inlineStr">
+        <is>
+          <t>🗑️ 重置存檔（清除所有紀錄）</t>
+        </is>
+      </c>
+      <c r="C30" t="inlineStr">
+        <is>
+          <t>🗑️ 重置存檔（清除所有紀錄）</t>
+        </is>
+      </c>
+      <c r="D30" t="inlineStr">
+        <is>
+          <t>🗑️ 重置存檔（清除所有紀錄）</t>
+        </is>
+      </c>
+      <c r="E30" t="inlineStr">
+        <is>
+          <t>🗑️ 重置存檔（清除所有紀錄）</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
fix(ui): fix save record and cheat modal open bugs and unify save diskette icon to monochrome theme SVG
</commit_message>
<xml_diff>
--- a/game_specs.xlsx
+++ b/game_specs.xlsx
@@ -3685,22 +3685,22 @@
       </c>
       <c r="B26" t="inlineStr">
         <is>
-          <t>💾 存檔紀錄</t>
+          <t>存檔紀錄</t>
         </is>
       </c>
       <c r="C26" t="inlineStr">
         <is>
-          <t>💾 存檔紀錄</t>
+          <t>存檔紀錄</t>
         </is>
       </c>
       <c r="D26" t="inlineStr">
         <is>
-          <t>💾 存檔紀錄</t>
+          <t>存檔紀錄</t>
         </is>
       </c>
       <c r="E26" t="inlineStr">
         <is>
-          <t>💾 存檔紀錄</t>
+          <t>存檔紀錄</t>
         </is>
       </c>
     </row>
@@ -3712,22 +3712,22 @@
       </c>
       <c r="B27" t="inlineStr">
         <is>
-          <t>💾 存檔紀錄與種子碼管理</t>
+          <t>存檔紀錄與種子碼管理</t>
         </is>
       </c>
       <c r="C27" t="inlineStr">
         <is>
-          <t>💾 存檔紀錄與種子碼管理</t>
+          <t>存檔紀錄與種子碼管理</t>
         </is>
       </c>
       <c r="D27" t="inlineStr">
         <is>
-          <t>💾 存檔紀錄與種子碼管理</t>
+          <t>存檔紀錄與種子碼管理</t>
         </is>
       </c>
       <c r="E27" t="inlineStr">
         <is>
-          <t>💾 存檔紀錄與種子碼管理</t>
+          <t>存檔紀錄與種子碼管理</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
feat(ui): eliminate save modal emojis, add records view shortcut and sync hint, and document visual design rules in AGENTS.md
</commit_message>
<xml_diff>
--- a/game_specs.xlsx
+++ b/game_specs.xlsx
@@ -3739,22 +3739,22 @@
       </c>
       <c r="B28" t="inlineStr">
         <is>
-          <t>📋 複製種子碼</t>
+          <t>複製種子碼</t>
         </is>
       </c>
       <c r="C28" t="inlineStr">
         <is>
-          <t>📋 複製種子碼</t>
+          <t>複製種子碼</t>
         </is>
       </c>
       <c r="D28" t="inlineStr">
         <is>
-          <t>📋 複製種子碼</t>
+          <t>複製種子碼</t>
         </is>
       </c>
       <c r="E28" t="inlineStr">
         <is>
-          <t>📋 複製種子碼</t>
+          <t>複製種子碼</t>
         </is>
       </c>
     </row>
@@ -3766,22 +3766,22 @@
       </c>
       <c r="B29" t="inlineStr">
         <is>
-          <t>📥 載入並套用種子碼</t>
+          <t>載入並套用種子碼</t>
         </is>
       </c>
       <c r="C29" t="inlineStr">
         <is>
-          <t>📥 載入並套用種子碼</t>
+          <t>載入並套用種子碼</t>
         </is>
       </c>
       <c r="D29" t="inlineStr">
         <is>
-          <t>📥 載入並套用種子碼</t>
+          <t>載入並套用種子碼</t>
         </is>
       </c>
       <c r="E29" t="inlineStr">
         <is>
-          <t>📥 載入並套用種子碼</t>
+          <t>載入並套用種子碼</t>
         </is>
       </c>
     </row>
@@ -3793,22 +3793,22 @@
       </c>
       <c r="B30" t="inlineStr">
         <is>
-          <t>🗑️ 重置存檔（清除所有紀錄）</t>
+          <t>重置存檔（清除所有紀錄）</t>
         </is>
       </c>
       <c r="C30" t="inlineStr">
         <is>
-          <t>🗑️ 重置存檔（清除所有紀錄）</t>
+          <t>重置存檔（清除所有紀錄）</t>
         </is>
       </c>
       <c r="D30" t="inlineStr">
         <is>
-          <t>🗑️ 重置存檔（清除所有紀錄）</t>
+          <t>重置存檔（清除所有紀錄）</t>
         </is>
       </c>
       <c r="E30" t="inlineStr">
         <is>
-          <t>🗑️ 重置存檔（清除所有紀錄）</t>
+          <t>重置存檔（清除所有紀錄）</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
feat(v0.3.0): add favicon.ico & favicon.svg, add footer version 0.3.0, fix mobile 0-latency QTE pointerdown, fix iOS audio resume, and button tactile feedback
</commit_message>
<xml_diff>
--- a/game_specs.xlsx
+++ b/game_specs.xlsx
@@ -10,7 +10,8 @@
     <sheet name="成長與數值公式" sheetId="6" r:id="rId6"/>
     <sheet name="切西瓜與圖鑑" sheetId="7" r:id="rId7"/>
     <sheet name="存檔與作弊管理" sheetId="8" r:id="rId8"/>
-    <sheet name="在地化字典" sheetId="9" r:id="rId9"/>
+    <sheet name="修練場與戰鬥日誌" sheetId="9" r:id="rId9"/>
+    <sheet name="在地化字典" sheetId="10" r:id="rId10"/>
   </sheets>
 </workbook>
 </file>
@@ -413,6 +414,1012 @@
 </worksheet>
 </file>
 
+<file path=xl/worksheets/sheet10.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetData>
+    <row r="1">
+      <c r="A1" t="inlineStr">
+        <is>
+          <t>鍵路徑</t>
+        </is>
+      </c>
+      <c r="B1" t="inlineStr">
+        <is>
+          <t>繁體中文 (zh-Hant)</t>
+        </is>
+      </c>
+      <c r="C1" t="inlineStr">
+        <is>
+          <t>簡體中文 (zh-Hans)</t>
+        </is>
+      </c>
+      <c r="D1" t="inlineStr">
+        <is>
+          <t>English (en)</t>
+        </is>
+      </c>
+      <c r="E1" t="inlineStr">
+        <is>
+          <t>日本語 (ja)</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>nav.home</t>
+        </is>
+      </c>
+      <c r="B2" t="inlineStr">
+        <is>
+          <t>nav.home</t>
+        </is>
+      </c>
+      <c r="C2" t="inlineStr">
+        <is>
+          <t>nav.home</t>
+        </is>
+      </c>
+      <c r="D2" t="inlineStr">
+        <is>
+          <t>nav.home</t>
+        </is>
+      </c>
+      <c r="E2" t="inlineStr">
+        <is>
+          <t>nav.home</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>nav.stages</t>
+        </is>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>nav.stages</t>
+        </is>
+      </c>
+      <c r="C3" t="inlineStr">
+        <is>
+          <t>nav.stages</t>
+        </is>
+      </c>
+      <c r="D3" t="inlineStr">
+        <is>
+          <t>nav.stages</t>
+        </is>
+      </c>
+      <c r="E3" t="inlineStr">
+        <is>
+          <t>nav.stages</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>nav.shop</t>
+        </is>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>nav.shop</t>
+        </is>
+      </c>
+      <c r="C4" t="inlineStr">
+        <is>
+          <t>nav.shop</t>
+        </is>
+      </c>
+      <c r="D4" t="inlineStr">
+        <is>
+          <t>nav.shop</t>
+        </is>
+      </c>
+      <c r="E4" t="inlineStr">
+        <is>
+          <t>nav.shop</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>nav.paperdoll</t>
+        </is>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>nav.paperdoll</t>
+        </is>
+      </c>
+      <c r="C5" t="inlineStr">
+        <is>
+          <t>nav.paperdoll</t>
+        </is>
+      </c>
+      <c r="D5" t="inlineStr">
+        <is>
+          <t>nav.paperdoll</t>
+        </is>
+      </c>
+      <c r="E5" t="inlineStr">
+        <is>
+          <t>nav.paperdoll</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>nav.growth</t>
+        </is>
+      </c>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>nav.growth</t>
+        </is>
+      </c>
+      <c r="C6" t="inlineStr">
+        <is>
+          <t>nav.growth</t>
+        </is>
+      </c>
+      <c r="D6" t="inlineStr">
+        <is>
+          <t>nav.growth</t>
+        </is>
+      </c>
+      <c r="E6" t="inlineStr">
+        <is>
+          <t>nav.growth</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>nav.gallery</t>
+        </is>
+      </c>
+      <c r="B7" t="inlineStr">
+        <is>
+          <t>nav.gallery</t>
+        </is>
+      </c>
+      <c r="C7" t="inlineStr">
+        <is>
+          <t>nav.gallery</t>
+        </is>
+      </c>
+      <c r="D7" t="inlineStr">
+        <is>
+          <t>nav.gallery</t>
+        </is>
+      </c>
+      <c r="E7" t="inlineStr">
+        <is>
+          <t>nav.gallery</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>nav.records</t>
+        </is>
+      </c>
+      <c r="B8" t="inlineStr">
+        <is>
+          <t>nav.records</t>
+        </is>
+      </c>
+      <c r="C8" t="inlineStr">
+        <is>
+          <t>nav.records</t>
+        </is>
+      </c>
+      <c r="D8" t="inlineStr">
+        <is>
+          <t>nav.records</t>
+        </is>
+      </c>
+      <c r="E8" t="inlineStr">
+        <is>
+          <t>nav.records</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>nav.guide</t>
+        </is>
+      </c>
+      <c r="B9" t="inlineStr">
+        <is>
+          <t>nav.guide</t>
+        </is>
+      </c>
+      <c r="C9" t="inlineStr">
+        <is>
+          <t>nav.guide</t>
+        </is>
+      </c>
+      <c r="D9" t="inlineStr">
+        <is>
+          <t>nav.guide</t>
+        </is>
+      </c>
+      <c r="E9" t="inlineStr">
+        <is>
+          <t>nav.guide</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
+        <is>
+          <t>nav.dojo</t>
+        </is>
+      </c>
+      <c r="B10" t="inlineStr">
+        <is>
+          <t>nav.dojo</t>
+        </is>
+      </c>
+      <c r="C10" t="inlineStr">
+        <is>
+          <t>nav.dojo</t>
+        </is>
+      </c>
+      <c r="D10" t="inlineStr">
+        <is>
+          <t>nav.dojo</t>
+        </is>
+      </c>
+      <c r="E10" t="inlineStr">
+        <is>
+          <t>nav.dojo</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="inlineStr">
+        <is>
+          <t>hands.rock</t>
+        </is>
+      </c>
+      <c r="B11" t="inlineStr">
+        <is>
+          <t>[object Object]</t>
+        </is>
+      </c>
+      <c r="C11" t="inlineStr">
+        <is>
+          <t>[object Object]</t>
+        </is>
+      </c>
+      <c r="D11" t="inlineStr">
+        <is>
+          <t>[object Object]</t>
+        </is>
+      </c>
+      <c r="E11" t="inlineStr">
+        <is>
+          <t>[object Object]</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="inlineStr">
+        <is>
+          <t>hands.paper</t>
+        </is>
+      </c>
+      <c r="B12" t="inlineStr">
+        <is>
+          <t>[object Object]</t>
+        </is>
+      </c>
+      <c r="C12" t="inlineStr">
+        <is>
+          <t>[object Object]</t>
+        </is>
+      </c>
+      <c r="D12" t="inlineStr">
+        <is>
+          <t>[object Object]</t>
+        </is>
+      </c>
+      <c r="E12" t="inlineStr">
+        <is>
+          <t>[object Object]</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="inlineStr">
+        <is>
+          <t>hands.scissors</t>
+        </is>
+      </c>
+      <c r="B13" t="inlineStr">
+        <is>
+          <t>[object Object]</t>
+        </is>
+      </c>
+      <c r="C13" t="inlineStr">
+        <is>
+          <t>[object Object]</t>
+        </is>
+      </c>
+      <c r="D13" t="inlineStr">
+        <is>
+          <t>[object Object]</t>
+        </is>
+      </c>
+      <c r="E13" t="inlineStr">
+        <is>
+          <t>[object Object]</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="inlineStr">
+        <is>
+          <t>dialogue.chant3</t>
+        </is>
+      </c>
+      <c r="B14" t="inlineStr">
+        <is>
+          <t>剪刀</t>
+        </is>
+      </c>
+      <c r="C14" t="inlineStr">
+        <is>
+          <t>剪刀</t>
+        </is>
+      </c>
+      <c r="D14" t="inlineStr">
+        <is>
+          <t>剪刀</t>
+        </is>
+      </c>
+      <c r="E14" t="inlineStr">
+        <is>
+          <t>剪刀</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" t="inlineStr">
+        <is>
+          <t>dialogue.chant2</t>
+        </is>
+      </c>
+      <c r="B15" t="inlineStr">
+        <is>
+          <t>石頭</t>
+        </is>
+      </c>
+      <c r="C15" t="inlineStr">
+        <is>
+          <t>石頭</t>
+        </is>
+      </c>
+      <c r="D15" t="inlineStr">
+        <is>
+          <t>石頭</t>
+        </is>
+      </c>
+      <c r="E15" t="inlineStr">
+        <is>
+          <t>石頭</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" t="inlineStr">
+        <is>
+          <t>dialogue.chant1</t>
+        </is>
+      </c>
+      <c r="B16" t="inlineStr">
+        <is>
+          <t>布！</t>
+        </is>
+      </c>
+      <c r="C16" t="inlineStr">
+        <is>
+          <t>布！</t>
+        </is>
+      </c>
+      <c r="D16" t="inlineStr">
+        <is>
+          <t>布！</t>
+        </is>
+      </c>
+      <c r="E16" t="inlineStr">
+        <is>
+          <t>布！</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" t="inlineStr">
+        <is>
+          <t>dialogue.morphReaction</t>
+        </is>
+      </c>
+      <c r="B17" t="inlineStr">
+        <is>
+          <t>咦……在最後一瞬間變拳了？</t>
+        </is>
+      </c>
+      <c r="C17" t="inlineStr">
+        <is>
+          <t>咦……在最後一瞬間變拳了？</t>
+        </is>
+      </c>
+      <c r="D17" t="inlineStr">
+        <is>
+          <t>咦……在最後一瞬間變拳了？</t>
+        </is>
+      </c>
+      <c r="E17" t="inlineStr">
+        <is>
+          <t>咦……在最後一瞬間變拳了？</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" t="inlineStr">
+        <is>
+          <t>ui.autoBattle</t>
+        </is>
+      </c>
+      <c r="B18" t="inlineStr">
+        <is>
+          <t>ui.autoBattle</t>
+        </is>
+      </c>
+      <c r="C18" t="inlineStr">
+        <is>
+          <t>ui.autoBattle</t>
+        </is>
+      </c>
+      <c r="D18" t="inlineStr">
+        <is>
+          <t>ui.autoBattle</t>
+        </is>
+      </c>
+      <c r="E18" t="inlineStr">
+        <is>
+          <t>ui.autoBattle</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" t="inlineStr">
+        <is>
+          <t>ui.autoWatermelonStock</t>
+        </is>
+      </c>
+      <c r="B19" t="inlineStr">
+        <is>
+          <t>累計切西瓜次數：5 / 999</t>
+        </is>
+      </c>
+      <c r="C19" t="inlineStr">
+        <is>
+          <t>累計切西瓜次數：5 / 999</t>
+        </is>
+      </c>
+      <c r="D19" t="inlineStr">
+        <is>
+          <t>累計切西瓜次數：5 / 999</t>
+        </is>
+      </c>
+      <c r="E19" t="inlineStr">
+        <is>
+          <t>累計切西瓜次數：5 / 999</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" t="inlineStr">
+        <is>
+          <t>ui.btnNextWatermelonRound</t>
+        </is>
+      </c>
+      <c r="B20" t="inlineStr">
+        <is>
+          <t>進行下一輪切西瓜 (剩餘 5)</t>
+        </is>
+      </c>
+      <c r="C20" t="inlineStr">
+        <is>
+          <t>進行下一輪切西瓜 (剩餘 5)</t>
+        </is>
+      </c>
+      <c r="D20" t="inlineStr">
+        <is>
+          <t>進行下一輪切西瓜 (剩餘 5)</t>
+        </is>
+      </c>
+      <c r="E20" t="inlineStr">
+        <is>
+          <t>進行下一輪切西瓜 (剩餘 5)</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" t="inlineStr">
+        <is>
+          <t>ui.floatingWatermelonTitle</t>
+        </is>
+      </c>
+      <c r="B21" t="inlineStr">
+        <is>
+          <t>🍉 蒙眼切西瓜 (自動刷關累積)</t>
+        </is>
+      </c>
+      <c r="C21" t="inlineStr">
+        <is>
+          <t>🍉 蒙眼切西瓜 (自動刷關累積)</t>
+        </is>
+      </c>
+      <c r="D21" t="inlineStr">
+        <is>
+          <t>🍉 蒙眼切西瓜 (自動刷關累積)</t>
+        </is>
+      </c>
+      <c r="E21" t="inlineStr">
+        <is>
+          <t>🍉 蒙眼切西瓜 (自動刷關累積)</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" t="inlineStr">
+        <is>
+          <t>ui.clearAll</t>
+        </is>
+      </c>
+      <c r="B22" t="inlineStr">
+        <is>
+          <t>ui.clearAll</t>
+        </is>
+      </c>
+      <c r="C22" t="inlineStr">
+        <is>
+          <t>ui.clearAll</t>
+        </is>
+      </c>
+      <c r="D22" t="inlineStr">
+        <is>
+          <t>ui.clearAll</t>
+        </is>
+      </c>
+      <c r="E22" t="inlineStr">
+        <is>
+          <t>ui.clearAll</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" t="inlineStr">
+        <is>
+          <t>ui.equip</t>
+        </is>
+      </c>
+      <c r="B23" t="inlineStr">
+        <is>
+          <t>ui.equip</t>
+        </is>
+      </c>
+      <c r="C23" t="inlineStr">
+        <is>
+          <t>ui.equip</t>
+        </is>
+      </c>
+      <c r="D23" t="inlineStr">
+        <is>
+          <t>ui.equip</t>
+        </is>
+      </c>
+      <c r="E23" t="inlineStr">
+        <is>
+          <t>ui.equip</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" t="inlineStr">
+        <is>
+          <t>ui.unequip</t>
+        </is>
+      </c>
+      <c r="B24" t="inlineStr">
+        <is>
+          <t>ui.unequip</t>
+        </is>
+      </c>
+      <c r="C24" t="inlineStr">
+        <is>
+          <t>ui.unequip</t>
+        </is>
+      </c>
+      <c r="D24" t="inlineStr">
+        <is>
+          <t>ui.unequip</t>
+        </is>
+      </c>
+      <c r="E24" t="inlineStr">
+        <is>
+          <t>ui.unequip</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" t="inlineStr">
+        <is>
+          <t>ui.victory</t>
+        </is>
+      </c>
+      <c r="B25" t="inlineStr">
+        <is>
+          <t>ui.victory</t>
+        </is>
+      </c>
+      <c r="C25" t="inlineStr">
+        <is>
+          <t>ui.victory</t>
+        </is>
+      </c>
+      <c r="D25" t="inlineStr">
+        <is>
+          <t>ui.victory</t>
+        </is>
+      </c>
+      <c r="E25" t="inlineStr">
+        <is>
+          <t>ui.victory</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" t="inlineStr">
+        <is>
+          <t>ui.defeat</t>
+        </is>
+      </c>
+      <c r="B26" t="inlineStr">
+        <is>
+          <t>ui.defeat</t>
+        </is>
+      </c>
+      <c r="C26" t="inlineStr">
+        <is>
+          <t>ui.defeat</t>
+        </is>
+      </c>
+      <c r="D26" t="inlineStr">
+        <is>
+          <t>ui.defeat</t>
+        </is>
+      </c>
+      <c r="E26" t="inlineStr">
+        <is>
+          <t>ui.defeat</t>
+        </is>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" t="inlineStr">
+        <is>
+          <t>ui.saveRecord</t>
+        </is>
+      </c>
+      <c r="B27" t="inlineStr">
+        <is>
+          <t>存檔紀錄</t>
+        </is>
+      </c>
+      <c r="C27" t="inlineStr">
+        <is>
+          <t>存檔紀錄</t>
+        </is>
+      </c>
+      <c r="D27" t="inlineStr">
+        <is>
+          <t>存檔紀錄</t>
+        </is>
+      </c>
+      <c r="E27" t="inlineStr">
+        <is>
+          <t>存檔紀錄</t>
+        </is>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" t="inlineStr">
+        <is>
+          <t>ui.saveRecordModalTitle</t>
+        </is>
+      </c>
+      <c r="B28" t="inlineStr">
+        <is>
+          <t>存檔紀錄與種子碼管理</t>
+        </is>
+      </c>
+      <c r="C28" t="inlineStr">
+        <is>
+          <t>存檔紀錄與種子碼管理</t>
+        </is>
+      </c>
+      <c r="D28" t="inlineStr">
+        <is>
+          <t>存檔紀錄與種子碼管理</t>
+        </is>
+      </c>
+      <c r="E28" t="inlineStr">
+        <is>
+          <t>存檔紀錄與種子碼管理</t>
+        </is>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" t="inlineStr">
+        <is>
+          <t>ui.btnCopySaveSeed</t>
+        </is>
+      </c>
+      <c r="B29" t="inlineStr">
+        <is>
+          <t>複製種子碼</t>
+        </is>
+      </c>
+      <c r="C29" t="inlineStr">
+        <is>
+          <t>複製種子碼</t>
+        </is>
+      </c>
+      <c r="D29" t="inlineStr">
+        <is>
+          <t>複製種子碼</t>
+        </is>
+      </c>
+      <c r="E29" t="inlineStr">
+        <is>
+          <t>複製種子碼</t>
+        </is>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" t="inlineStr">
+        <is>
+          <t>ui.btnImportSaveSeed</t>
+        </is>
+      </c>
+      <c r="B30" t="inlineStr">
+        <is>
+          <t>載入並套用種子碼</t>
+        </is>
+      </c>
+      <c r="C30" t="inlineStr">
+        <is>
+          <t>載入並套用種子碼</t>
+        </is>
+      </c>
+      <c r="D30" t="inlineStr">
+        <is>
+          <t>載入並套用種子碼</t>
+        </is>
+      </c>
+      <c r="E30" t="inlineStr">
+        <is>
+          <t>載入並套用種子碼</t>
+        </is>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" t="inlineStr">
+        <is>
+          <t>ui.btnModalResetSave</t>
+        </is>
+      </c>
+      <c r="B31" t="inlineStr">
+        <is>
+          <t>重置存檔（清除所有紀錄）</t>
+        </is>
+      </c>
+      <c r="C31" t="inlineStr">
+        <is>
+          <t>重置存檔（清除所有紀錄）</t>
+        </is>
+      </c>
+      <c r="D31" t="inlineStr">
+        <is>
+          <t>重置存檔（清除所有紀錄）</t>
+        </is>
+      </c>
+      <c r="E31" t="inlineStr">
+        <is>
+          <t>重置存檔（清除所有紀錄）</t>
+        </is>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" t="inlineStr">
+        <is>
+          <t>dojo.title</t>
+        </is>
+      </c>
+      <c r="B32" t="inlineStr">
+        <is>
+          <t>dojo.title</t>
+        </is>
+      </c>
+      <c r="C32" t="inlineStr">
+        <is>
+          <t>dojo.title</t>
+        </is>
+      </c>
+      <c r="D32" t="inlineStr">
+        <is>
+          <t>dojo.title</t>
+        </is>
+      </c>
+      <c r="E32" t="inlineStr">
+        <is>
+          <t>dojo.title</t>
+        </is>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" t="inlineStr">
+        <is>
+          <t>dojo.mode1Title</t>
+        </is>
+      </c>
+      <c r="B33" t="inlineStr">
+        <is>
+          <t>模式一：純 QTE 無限反應練習</t>
+        </is>
+      </c>
+      <c r="C33" t="inlineStr">
+        <is>
+          <t>模式一：純 QTE 無限反應練習</t>
+        </is>
+      </c>
+      <c r="D33" t="inlineStr">
+        <is>
+          <t>模式一：純 QTE 無限反應練習</t>
+        </is>
+      </c>
+      <c r="E33" t="inlineStr">
+        <is>
+          <t>模式一：純 QTE 無限反應練習</t>
+        </is>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" t="inlineStr">
+        <is>
+          <t>dojo.mode2Title</t>
+        </is>
+      </c>
+      <c r="B34" t="inlineStr">
+        <is>
+          <t>模式二：戰鬥模擬與 DPS 測試沙盒</t>
+        </is>
+      </c>
+      <c r="C34" t="inlineStr">
+        <is>
+          <t>模式二：戰鬥模擬與 DPS 測試沙盒</t>
+        </is>
+      </c>
+      <c r="D34" t="inlineStr">
+        <is>
+          <t>模式二：戰鬥模擬與 DPS 測試沙盒</t>
+        </is>
+      </c>
+      <c r="E34" t="inlineStr">
+        <is>
+          <t>模式二：戰鬥模擬與 DPS 測試沙盒</t>
+        </is>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" t="inlineStr">
+        <is>
+          <t>ui.recentDamageLog</t>
+        </is>
+      </c>
+      <c r="B35" t="inlineStr">
+        <is>
+          <t>最近傷害</t>
+        </is>
+      </c>
+      <c r="C35" t="inlineStr">
+        <is>
+          <t>最近傷害</t>
+        </is>
+      </c>
+      <c r="D35" t="inlineStr">
+        <is>
+          <t>最近傷害</t>
+        </is>
+      </c>
+      <c r="E35" t="inlineStr">
+        <is>
+          <t>最近傷害</t>
+        </is>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" t="inlineStr">
+        <is>
+          <t>ui.playerAtk</t>
+        </is>
+      </c>
+      <c r="B36" t="inlineStr">
+        <is>
+          <t>ui.playerAtk</t>
+        </is>
+      </c>
+      <c r="C36" t="inlineStr">
+        <is>
+          <t>ui.playerAtk</t>
+        </is>
+      </c>
+      <c r="D36" t="inlineStr">
+        <is>
+          <t>ui.playerAtk</t>
+        </is>
+      </c>
+      <c r="E36" t="inlineStr">
+        <is>
+          <t>ui.playerAtk</t>
+        </is>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" t="inlineStr">
+        <is>
+          <t>ui.enemyAtk</t>
+        </is>
+      </c>
+      <c r="B37" t="inlineStr">
+        <is>
+          <t>ui.enemyAtk</t>
+        </is>
+      </c>
+      <c r="C37" t="inlineStr">
+        <is>
+          <t>ui.enemyAtk</t>
+        </is>
+      </c>
+      <c r="D37" t="inlineStr">
+        <is>
+          <t>ui.enemyAtk</t>
+        </is>
+      </c>
+      <c r="E37" t="inlineStr">
+        <is>
+          <t>ui.enemyAtk</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+</worksheet>
+</file>
+
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetData>
@@ -3005,810 +4012,210 @@
     <row r="1">
       <c r="A1" t="inlineStr">
         <is>
-          <t>鍵路徑</t>
+          <t>模式代碼</t>
         </is>
       </c>
       <c r="B1" t="inlineStr">
         <is>
-          <t>繁體中文 (zh-Hant)</t>
+          <t>模式名稱</t>
         </is>
       </c>
       <c r="C1" t="inlineStr">
         <is>
-          <t>簡體中文 (zh-Hans)</t>
+          <t>式別</t>
         </is>
       </c>
       <c r="D1" t="inlineStr">
         <is>
-          <t>English (en)</t>
+          <t>式別名稱</t>
         </is>
       </c>
       <c r="E1" t="inlineStr">
         <is>
-          <t>日本語 (ja)</t>
+          <t>對手外觀</t>
+        </is>
+      </c>
+      <c r="F1" t="inlineStr">
+        <is>
+          <t>預設生命(HP)</t>
+        </is>
+      </c>
+      <c r="G1" t="inlineStr">
+        <is>
+          <t>預設傷害(ATK)</t>
+        </is>
+      </c>
+      <c r="H1" t="inlineStr">
+        <is>
+          <t>機制與用途說明</t>
         </is>
       </c>
     </row>
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>nav.home</t>
+          <t>mode1</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>nav.home</t>
+          <t>模式一：純 QTE 反應練習</t>
         </is>
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>nav.home</t>
+          <t>style1</t>
         </is>
       </c>
       <c r="D2" t="inlineStr">
         <is>
-          <t>nav.home</t>
+          <t>第一式：單軌疾速</t>
         </is>
       </c>
       <c r="E2" t="inlineStr">
         <is>
-          <t>nav.home</t>
+          <t>無（純 QTE 軌道）</t>
+        </is>
+      </c>
+      <c r="F2" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="G2" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="H2" t="inlineStr">
+        <is>
+          <t>8 方向單軌連續輸入，統計連擊數 (Combo)、最高連擊、平均反應時間 (ms) 與成功率</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>nav.stages</t>
+          <t>mode1</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>nav.stages</t>
+          <t>模式一：純 QTE 反應練習</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>nav.stages</t>
+          <t>style2</t>
         </is>
       </c>
       <c r="D3" t="inlineStr">
         <is>
-          <t>nav.stages</t>
+          <t>第二式：雙軌協同</t>
         </is>
       </c>
       <c r="E3" t="inlineStr">
         <is>
-          <t>nav.stages</t>
+          <t>無（雙 QTE 軌道）</t>
+        </is>
+      </c>
+      <c r="F3" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="G3" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="H3" t="inlineStr">
+        <is>
+          <t>雙手雙軌獨立判定（左手 WASD、右手 方向鍵），模擬終章極限鍵位</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>nav.shop</t>
+          <t>mode2</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>nav.shop</t>
+          <t>模式二：戰鬥沙盒與 DPS 測試</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>nav.shop</t>
+          <t>style1</t>
         </is>
       </c>
       <c r="D4" t="inlineStr">
         <is>
-          <t>nav.shop</t>
+          <t>第一式：單體木樁</t>
         </is>
       </c>
       <c r="E4" t="inlineStr">
         <is>
-          <t>nav.shop</t>
+          <t>影・小樂（全黑剪影）</t>
+        </is>
+      </c>
+      <c r="F4" t="inlineStr">
+        <is>
+          <t>10,000 (可自訂 1~999,999)</t>
+        </is>
+      </c>
+      <c r="G4" t="inlineStr">
+        <is>
+          <t>0 (可自訂傷害)</t>
+        </is>
+      </c>
+      <c r="H4" t="inlineStr">
+        <is>
+          <t>標準 3-2-1 猜拳、變拳、摸摸與 QTE 反制，無敗北壓力，測試配裝實戰 DPS</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>nav.paperdoll</t>
+          <t>mode2</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>nav.paperdoll</t>
+          <t>模式二：戰鬥沙盒與 DPS 測試</t>
         </is>
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>nav.paperdoll</t>
+          <t>style2</t>
         </is>
       </c>
       <c r="D5" t="inlineStr">
         <is>
-          <t>nav.paperdoll</t>
+          <t>第二式：雙生木樁</t>
         </is>
       </c>
       <c r="E5" t="inlineStr">
         <is>
-          <t>nav.paperdoll</t>
-        </is>
-      </c>
-    </row>
-    <row r="6">
-      <c r="A6" t="inlineStr">
-        <is>
-          <t>nav.growth</t>
-        </is>
-      </c>
-      <c r="B6" t="inlineStr">
-        <is>
-          <t>nav.growth</t>
-        </is>
-      </c>
-      <c r="C6" t="inlineStr">
-        <is>
-          <t>nav.growth</t>
-        </is>
-      </c>
-      <c r="D6" t="inlineStr">
-        <is>
-          <t>nav.growth</t>
-        </is>
-      </c>
-      <c r="E6" t="inlineStr">
-        <is>
-          <t>nav.growth</t>
-        </is>
-      </c>
-    </row>
-    <row r="7">
-      <c r="A7" t="inlineStr">
-        <is>
-          <t>nav.gallery</t>
-        </is>
-      </c>
-      <c r="B7" t="inlineStr">
-        <is>
-          <t>nav.gallery</t>
-        </is>
-      </c>
-      <c r="C7" t="inlineStr">
-        <is>
-          <t>nav.gallery</t>
-        </is>
-      </c>
-      <c r="D7" t="inlineStr">
-        <is>
-          <t>nav.gallery</t>
-        </is>
-      </c>
-      <c r="E7" t="inlineStr">
-        <is>
-          <t>nav.gallery</t>
-        </is>
-      </c>
-    </row>
-    <row r="8">
-      <c r="A8" t="inlineStr">
-        <is>
-          <t>nav.records</t>
-        </is>
-      </c>
-      <c r="B8" t="inlineStr">
-        <is>
-          <t>nav.records</t>
-        </is>
-      </c>
-      <c r="C8" t="inlineStr">
-        <is>
-          <t>nav.records</t>
-        </is>
-      </c>
-      <c r="D8" t="inlineStr">
-        <is>
-          <t>nav.records</t>
-        </is>
-      </c>
-      <c r="E8" t="inlineStr">
-        <is>
-          <t>nav.records</t>
-        </is>
-      </c>
-    </row>
-    <row r="9">
-      <c r="A9" t="inlineStr">
-        <is>
-          <t>nav.guide</t>
-        </is>
-      </c>
-      <c r="B9" t="inlineStr">
-        <is>
-          <t>nav.guide</t>
-        </is>
-      </c>
-      <c r="C9" t="inlineStr">
-        <is>
-          <t>nav.guide</t>
-        </is>
-      </c>
-      <c r="D9" t="inlineStr">
-        <is>
-          <t>nav.guide</t>
-        </is>
-      </c>
-      <c r="E9" t="inlineStr">
-        <is>
-          <t>nav.guide</t>
-        </is>
-      </c>
-    </row>
-    <row r="10">
-      <c r="A10" t="inlineStr">
-        <is>
-          <t>hands.rock</t>
-        </is>
-      </c>
-      <c r="B10" t="inlineStr">
-        <is>
-          <t>[object Object]</t>
-        </is>
-      </c>
-      <c r="C10" t="inlineStr">
-        <is>
-          <t>[object Object]</t>
-        </is>
-      </c>
-      <c r="D10" t="inlineStr">
-        <is>
-          <t>[object Object]</t>
-        </is>
-      </c>
-      <c r="E10" t="inlineStr">
-        <is>
-          <t>[object Object]</t>
-        </is>
-      </c>
-    </row>
-    <row r="11">
-      <c r="A11" t="inlineStr">
-        <is>
-          <t>hands.paper</t>
-        </is>
-      </c>
-      <c r="B11" t="inlineStr">
-        <is>
-          <t>[object Object]</t>
-        </is>
-      </c>
-      <c r="C11" t="inlineStr">
-        <is>
-          <t>[object Object]</t>
-        </is>
-      </c>
-      <c r="D11" t="inlineStr">
-        <is>
-          <t>[object Object]</t>
-        </is>
-      </c>
-      <c r="E11" t="inlineStr">
-        <is>
-          <t>[object Object]</t>
-        </is>
-      </c>
-    </row>
-    <row r="12">
-      <c r="A12" t="inlineStr">
-        <is>
-          <t>hands.scissors</t>
-        </is>
-      </c>
-      <c r="B12" t="inlineStr">
-        <is>
-          <t>[object Object]</t>
-        </is>
-      </c>
-      <c r="C12" t="inlineStr">
-        <is>
-          <t>[object Object]</t>
-        </is>
-      </c>
-      <c r="D12" t="inlineStr">
-        <is>
-          <t>[object Object]</t>
-        </is>
-      </c>
-      <c r="E12" t="inlineStr">
-        <is>
-          <t>[object Object]</t>
-        </is>
-      </c>
-    </row>
-    <row r="13">
-      <c r="A13" t="inlineStr">
-        <is>
-          <t>dialogue.chant3</t>
-        </is>
-      </c>
-      <c r="B13" t="inlineStr">
-        <is>
-          <t>剪刀</t>
-        </is>
-      </c>
-      <c r="C13" t="inlineStr">
-        <is>
-          <t>剪刀</t>
-        </is>
-      </c>
-      <c r="D13" t="inlineStr">
-        <is>
-          <t>剪刀</t>
-        </is>
-      </c>
-      <c r="E13" t="inlineStr">
-        <is>
-          <t>剪刀</t>
-        </is>
-      </c>
-    </row>
-    <row r="14">
-      <c r="A14" t="inlineStr">
-        <is>
-          <t>dialogue.chant2</t>
-        </is>
-      </c>
-      <c r="B14" t="inlineStr">
-        <is>
-          <t>石頭</t>
-        </is>
-      </c>
-      <c r="C14" t="inlineStr">
-        <is>
-          <t>石頭</t>
-        </is>
-      </c>
-      <c r="D14" t="inlineStr">
-        <is>
-          <t>石頭</t>
-        </is>
-      </c>
-      <c r="E14" t="inlineStr">
-        <is>
-          <t>石頭</t>
-        </is>
-      </c>
-    </row>
-    <row r="15">
-      <c r="A15" t="inlineStr">
-        <is>
-          <t>dialogue.chant1</t>
-        </is>
-      </c>
-      <c r="B15" t="inlineStr">
-        <is>
-          <t>布！</t>
-        </is>
-      </c>
-      <c r="C15" t="inlineStr">
-        <is>
-          <t>布！</t>
-        </is>
-      </c>
-      <c r="D15" t="inlineStr">
-        <is>
-          <t>布！</t>
-        </is>
-      </c>
-      <c r="E15" t="inlineStr">
-        <is>
-          <t>布！</t>
-        </is>
-      </c>
-    </row>
-    <row r="16">
-      <c r="A16" t="inlineStr">
-        <is>
-          <t>dialogue.morphReaction</t>
-        </is>
-      </c>
-      <c r="B16" t="inlineStr">
-        <is>
-          <t>咦……在最後一瞬間變拳了？</t>
-        </is>
-      </c>
-      <c r="C16" t="inlineStr">
-        <is>
-          <t>咦……在最後一瞬間變拳了？</t>
-        </is>
-      </c>
-      <c r="D16" t="inlineStr">
-        <is>
-          <t>咦……在最後一瞬間變拳了？</t>
-        </is>
-      </c>
-      <c r="E16" t="inlineStr">
-        <is>
-          <t>咦……在最後一瞬間變拳了？</t>
-        </is>
-      </c>
-    </row>
-    <row r="17">
-      <c r="A17" t="inlineStr">
-        <is>
-          <t>ui.autoBattle</t>
-        </is>
-      </c>
-      <c r="B17" t="inlineStr">
-        <is>
-          <t>ui.autoBattle</t>
-        </is>
-      </c>
-      <c r="C17" t="inlineStr">
-        <is>
-          <t>ui.autoBattle</t>
-        </is>
-      </c>
-      <c r="D17" t="inlineStr">
-        <is>
-          <t>ui.autoBattle</t>
-        </is>
-      </c>
-      <c r="E17" t="inlineStr">
-        <is>
-          <t>ui.autoBattle</t>
-        </is>
-      </c>
-    </row>
-    <row r="18">
-      <c r="A18" t="inlineStr">
-        <is>
-          <t>ui.autoWatermelonStock</t>
-        </is>
-      </c>
-      <c r="B18" t="inlineStr">
-        <is>
-          <t>累計切西瓜次數：5 / 999</t>
-        </is>
-      </c>
-      <c r="C18" t="inlineStr">
-        <is>
-          <t>累計切西瓜次數：5 / 999</t>
-        </is>
-      </c>
-      <c r="D18" t="inlineStr">
-        <is>
-          <t>累計切西瓜次數：5 / 999</t>
-        </is>
-      </c>
-      <c r="E18" t="inlineStr">
-        <is>
-          <t>累計切西瓜次數：5 / 999</t>
-        </is>
-      </c>
-    </row>
-    <row r="19">
-      <c r="A19" t="inlineStr">
-        <is>
-          <t>ui.btnNextWatermelonRound</t>
-        </is>
-      </c>
-      <c r="B19" t="inlineStr">
-        <is>
-          <t>進行下一輪切西瓜 (剩餘 5)</t>
-        </is>
-      </c>
-      <c r="C19" t="inlineStr">
-        <is>
-          <t>進行下一輪切西瓜 (剩餘 5)</t>
-        </is>
-      </c>
-      <c r="D19" t="inlineStr">
-        <is>
-          <t>進行下一輪切西瓜 (剩餘 5)</t>
-        </is>
-      </c>
-      <c r="E19" t="inlineStr">
-        <is>
-          <t>進行下一輪切西瓜 (剩餘 5)</t>
-        </is>
-      </c>
-    </row>
-    <row r="20">
-      <c r="A20" t="inlineStr">
-        <is>
-          <t>ui.floatingWatermelonTitle</t>
-        </is>
-      </c>
-      <c r="B20" t="inlineStr">
-        <is>
-          <t>🍉 蒙眼切西瓜 (自動刷關累積)</t>
-        </is>
-      </c>
-      <c r="C20" t="inlineStr">
-        <is>
-          <t>🍉 蒙眼切西瓜 (自動刷關累積)</t>
-        </is>
-      </c>
-      <c r="D20" t="inlineStr">
-        <is>
-          <t>🍉 蒙眼切西瓜 (自動刷關累積)</t>
-        </is>
-      </c>
-      <c r="E20" t="inlineStr">
-        <is>
-          <t>🍉 蒙眼切西瓜 (自動刷關累積)</t>
-        </is>
-      </c>
-    </row>
-    <row r="21">
-      <c r="A21" t="inlineStr">
-        <is>
-          <t>ui.clearAll</t>
-        </is>
-      </c>
-      <c r="B21" t="inlineStr">
-        <is>
-          <t>ui.clearAll</t>
-        </is>
-      </c>
-      <c r="C21" t="inlineStr">
-        <is>
-          <t>ui.clearAll</t>
-        </is>
-      </c>
-      <c r="D21" t="inlineStr">
-        <is>
-          <t>ui.clearAll</t>
-        </is>
-      </c>
-      <c r="E21" t="inlineStr">
-        <is>
-          <t>ui.clearAll</t>
-        </is>
-      </c>
-    </row>
-    <row r="22">
-      <c r="A22" t="inlineStr">
-        <is>
-          <t>ui.equip</t>
-        </is>
-      </c>
-      <c r="B22" t="inlineStr">
-        <is>
-          <t>ui.equip</t>
-        </is>
-      </c>
-      <c r="C22" t="inlineStr">
-        <is>
-          <t>ui.equip</t>
-        </is>
-      </c>
-      <c r="D22" t="inlineStr">
-        <is>
-          <t>ui.equip</t>
-        </is>
-      </c>
-      <c r="E22" t="inlineStr">
-        <is>
-          <t>ui.equip</t>
-        </is>
-      </c>
-    </row>
-    <row r="23">
-      <c r="A23" t="inlineStr">
-        <is>
-          <t>ui.unequip</t>
-        </is>
-      </c>
-      <c r="B23" t="inlineStr">
-        <is>
-          <t>ui.unequip</t>
-        </is>
-      </c>
-      <c r="C23" t="inlineStr">
-        <is>
-          <t>ui.unequip</t>
-        </is>
-      </c>
-      <c r="D23" t="inlineStr">
-        <is>
-          <t>ui.unequip</t>
-        </is>
-      </c>
-      <c r="E23" t="inlineStr">
-        <is>
-          <t>ui.unequip</t>
-        </is>
-      </c>
-    </row>
-    <row r="24">
-      <c r="A24" t="inlineStr">
-        <is>
-          <t>ui.victory</t>
-        </is>
-      </c>
-      <c r="B24" t="inlineStr">
-        <is>
-          <t>ui.victory</t>
-        </is>
-      </c>
-      <c r="C24" t="inlineStr">
-        <is>
-          <t>ui.victory</t>
-        </is>
-      </c>
-      <c r="D24" t="inlineStr">
-        <is>
-          <t>ui.victory</t>
-        </is>
-      </c>
-      <c r="E24" t="inlineStr">
-        <is>
-          <t>ui.victory</t>
-        </is>
-      </c>
-    </row>
-    <row r="25">
-      <c r="A25" t="inlineStr">
-        <is>
-          <t>ui.defeat</t>
-        </is>
-      </c>
-      <c r="B25" t="inlineStr">
-        <is>
-          <t>ui.defeat</t>
-        </is>
-      </c>
-      <c r="C25" t="inlineStr">
-        <is>
-          <t>ui.defeat</t>
-        </is>
-      </c>
-      <c r="D25" t="inlineStr">
-        <is>
-          <t>ui.defeat</t>
-        </is>
-      </c>
-      <c r="E25" t="inlineStr">
-        <is>
-          <t>ui.defeat</t>
-        </is>
-      </c>
-    </row>
-    <row r="26">
-      <c r="A26" t="inlineStr">
-        <is>
-          <t>ui.saveRecord</t>
-        </is>
-      </c>
-      <c r="B26" t="inlineStr">
-        <is>
-          <t>存檔紀錄</t>
-        </is>
-      </c>
-      <c r="C26" t="inlineStr">
-        <is>
-          <t>存檔紀錄</t>
-        </is>
-      </c>
-      <c r="D26" t="inlineStr">
-        <is>
-          <t>存檔紀錄</t>
-        </is>
-      </c>
-      <c r="E26" t="inlineStr">
-        <is>
-          <t>存檔紀錄</t>
-        </is>
-      </c>
-    </row>
-    <row r="27">
-      <c r="A27" t="inlineStr">
-        <is>
-          <t>ui.saveRecordModalTitle</t>
-        </is>
-      </c>
-      <c r="B27" t="inlineStr">
-        <is>
-          <t>存檔紀錄與種子碼管理</t>
-        </is>
-      </c>
-      <c r="C27" t="inlineStr">
-        <is>
-          <t>存檔紀錄與種子碼管理</t>
-        </is>
-      </c>
-      <c r="D27" t="inlineStr">
-        <is>
-          <t>存檔紀錄與種子碼管理</t>
-        </is>
-      </c>
-      <c r="E27" t="inlineStr">
-        <is>
-          <t>存檔紀錄與種子碼管理</t>
-        </is>
-      </c>
-    </row>
-    <row r="28">
-      <c r="A28" t="inlineStr">
-        <is>
-          <t>ui.btnCopySaveSeed</t>
-        </is>
-      </c>
-      <c r="B28" t="inlineStr">
-        <is>
-          <t>複製種子碼</t>
-        </is>
-      </c>
-      <c r="C28" t="inlineStr">
-        <is>
-          <t>複製種子碼</t>
-        </is>
-      </c>
-      <c r="D28" t="inlineStr">
-        <is>
-          <t>複製種子碼</t>
-        </is>
-      </c>
-      <c r="E28" t="inlineStr">
-        <is>
-          <t>複製種子碼</t>
-        </is>
-      </c>
-    </row>
-    <row r="29">
-      <c r="A29" t="inlineStr">
-        <is>
-          <t>ui.btnImportSaveSeed</t>
-        </is>
-      </c>
-      <c r="B29" t="inlineStr">
-        <is>
-          <t>載入並套用種子碼</t>
-        </is>
-      </c>
-      <c r="C29" t="inlineStr">
-        <is>
-          <t>載入並套用種子碼</t>
-        </is>
-      </c>
-      <c r="D29" t="inlineStr">
-        <is>
-          <t>載入並套用種子碼</t>
-        </is>
-      </c>
-      <c r="E29" t="inlineStr">
-        <is>
-          <t>載入並套用種子碼</t>
-        </is>
-      </c>
-    </row>
-    <row r="30">
-      <c r="A30" t="inlineStr">
-        <is>
-          <t>ui.btnModalResetSave</t>
-        </is>
-      </c>
-      <c r="B30" t="inlineStr">
-        <is>
-          <t>重置存檔（清除所有紀錄）</t>
-        </is>
-      </c>
-      <c r="C30" t="inlineStr">
-        <is>
-          <t>重置存檔（清除所有紀錄）</t>
-        </is>
-      </c>
-      <c r="D30" t="inlineStr">
-        <is>
-          <t>重置存檔（清除所有紀錄）</t>
-        </is>
-      </c>
-      <c r="E30" t="inlineStr">
-        <is>
-          <t>重置存檔（清除所有紀錄）</t>
+          <t>雙生影・小樂（全黑剪影）</t>
+        </is>
+      </c>
+      <c r="F5" t="inlineStr">
+        <is>
+          <t>20,000 (每隻 10,000 可自訂)</t>
+        </is>
+      </c>
+      <c r="G5" t="inlineStr">
+        <is>
+          <t>0 (可自訂傷害)</t>
+        </is>
+      </c>
+      <c r="H5" t="inlineStr">
+        <is>
+          <t>模擬第 4 關雙手出拳與雙軌 QTE，支援雙手解放技能實戰演練</t>
         </is>
       </c>
     </row>

</xml_diff>